<commit_message>
Add the 3 Sept 2026 revolution (season 2, 2 sets) and unstick the short-season axis label
</commit_message>
<xml_diff>
--- a/data/stats.xlsx
+++ b/data/stats.xlsx
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="104">
   <si>
     <t>Date</t>
   </si>
@@ -374,6 +374,9 @@
   </si>
   <si>
     <t>R20260725-1</t>
+  </si>
+  <si>
+    <t>R20260903-1</t>
   </si>
 </sst>
 </file>
@@ -803,7 +806,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.90625" customWidth="1"/>
@@ -3878,8 +3881,96 @@
         <v>101</v>
       </c>
     </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>103</v>
+      </c>
+      <c r="B33" s="1">
+        <v>46268</v>
+      </c>
+      <c r="F33" t="str" cm="1">
+        <f t="array" ref="F33">COUNTIFS(
+ Matches!$A$2:$A$200,$A33,
+ Matches!$I$2:$I$200,"*"&amp;F$1&amp;"*"
+)
+&amp;" ("&amp;
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A33) *
+ ((Matches!$C$2:$C$200=F$1)+(Matches!$D$2:$D$200=F$1)) *
+ Matches!$G$2:$G$200
+)
++
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A33) *
+ ((Matches!$E$2:$E$200=F$1)+(Matches!$F$2:$F$200=F$1)) *
+ Matches!$H$2:$H$200
+)
+&amp;")"</f>
+        <v>0 (14)</v>
+      </c>
+      <c r="G33" t="str" cm="1">
+        <f t="array" ref="G33">COUNTIFS(
+ Matches!$A$2:$A$200,$A33,
+ Matches!$I$2:$I$200,"*"&amp;G$1&amp;"*"
+)
+&amp;" ("&amp;
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A33) *
+ ((Matches!$C$2:$C$200=G$1)+(Matches!$D$2:$D$200=G$1)) *
+ Matches!$G$2:$G$200
+)
++
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A33) *
+ ((Matches!$E$2:$E$200=G$1)+(Matches!$F$2:$F$200=G$1)) *
+ Matches!$H$2:$H$200
+)
+&amp;")"</f>
+        <v>2 (20)</v>
+      </c>
+      <c r="H33" t="str" cm="1">
+        <f t="array" ref="H33">COUNTIFS(
+ Matches!$A$2:$A$200,$A33,
+ Matches!$I$2:$I$200,"*"&amp;H$1&amp;"*"
+)
+&amp;" ("&amp;
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A33) *
+ ((Matches!$C$2:$C$200=H$1)+(Matches!$D$2:$D$200=H$1)) *
+ Matches!$G$2:$G$200
+)
++
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A33) *
+ ((Matches!$E$2:$E$200=H$1)+(Matches!$F$2:$F$200=H$1)) *
+ Matches!$H$2:$H$200
+)
+&amp;")"</f>
+        <v>1 (18)</v>
+      </c>
+      <c r="I33" t="str" cm="1">
+        <f t="array" ref="I33">COUNTIFS(
+ Matches!$A$2:$A$200,$A33,
+ Matches!$I$2:$I$200,"*"&amp;I$1&amp;"*"
+)
+&amp;" ("&amp;
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A33) *
+ ((Matches!$C$2:$C$200=I$1)+(Matches!$D$2:$D$200=I$1)) *
+ Matches!$G$2:$G$200
+)
++
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A33) *
+ ((Matches!$E$2:$E$200=I$1)+(Matches!$F$2:$F$200=I$1)) *
+ Matches!$H$2:$H$200
+)
+&amp;")"</f>
+        <v>1 (16)</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:I32">
+  <conditionalFormatting sqref="F2:I33">
     <cfRule type="expression" dxfId="10" priority="1">
       <formula>LEFT(F2,1)="0"</formula>
     </cfRule>
@@ -3910,7 +4001,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6F95CC-DDBC-4D0D-92B0-0E6D3AF66C09}">
-  <dimension ref="A1:K93"/>
+  <dimension ref="A1:K95"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.90625" customWidth="1"/>
@@ -7196,6 +7287,80 @@
       <c r="K93" t="str">
         <f t="shared" si="2"/>
         <v>R20260725-1-3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>103</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>15</v>
+      </c>
+      <c r="D94" t="s">
+        <v>14</v>
+      </c>
+      <c r="E94" t="s">
+        <v>12</v>
+      </c>
+      <c r="F94" t="s">
+        <v>13</v>
+      </c>
+      <c r="G94" s="4">
+        <v>10</v>
+      </c>
+      <c r="H94" s="4">
+        <v>6</v>
+      </c>
+      <c r="I94" t="str">
+        <f>IF(G94&gt;H94,
+   IF(C94&lt;D94, C94&amp;"/"&amp;D94, D94&amp;"/"&amp;C94),
+   IF(E94&lt;F94, E94&amp;"/"&amp;F94, F94&amp;"/"&amp;E94)
+)</f>
+        <v>ML/MN</v>
+      </c>
+      <c r="K94" t="str">
+        <f>_xlfn.CONCAT(A94, "-", B94)</f>
+        <v>R20260903-1-1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>103</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95" t="s">
+        <v>15</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>12</v>
+      </c>
+      <c r="G95" s="4">
+        <v>10</v>
+      </c>
+      <c r="H95" s="4">
+        <v>8</v>
+      </c>
+      <c r="I95" t="str">
+        <f>IF(G95&gt;H95,
+   IF(C95&lt;D95, C95&amp;"/"&amp;D95, D95&amp;"/"&amp;C95),
+   IF(E95&lt;F95, E95&amp;"/"&amp;F95, F95&amp;"/"&amp;E95)
+)</f>
+        <v>ML/VM</v>
+      </c>
+      <c r="K95" t="str">
+        <f>_xlfn.CONCAT(A95, "-", B95)</f>
+        <v>R20260903-1-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>